<commit_message>
Balancete fechado em 15/10 (10º d.u.) e destaque dos processos em paralelo
- Imagem: raias mostrando o que corre em paralelo de 02/10 a 15/10
- Aba Fluxo no Tempo: contabilidade termina no balancete fechado (10º d.u.)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0125feEMvz8hWRDaMuVf6tsQ
</commit_message>
<xml_diff>
--- a/12. Ficha de Controle Grupo Comber - SETEMBRO 2026.xlsx
+++ b/12. Ficha de Controle Grupo Comber - SETEMBRO 2026.xlsx
@@ -13119,14 +13119,14 @@
     <tabColor rgb="FF2E75B6"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:S34"/>
+  <dimension ref="B2:O34"/>
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="2.5" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="19" width="8.2" customWidth="1"/>
-    <col min="20" max="20" width="2.5" customWidth="1"/>
+    <col min="4" max="15" width="9.5" customWidth="1"/>
+    <col min="16" max="16" width="2.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -13215,26 +13215,6 @@
           <t xml:space="preserve">11º d.u.</t>
         </is>
       </c>
-      <c r="P5" s="325" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12º d.u.</t>
-        </is>
-      </c>
-      <c r="Q5" s="325" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13º d.u.</t>
-        </is>
-      </c>
-      <c r="R5" s="325" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14º d.u.</t>
-        </is>
-      </c>
-      <c r="S5" s="325" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15º d.u.</t>
-        </is>
-      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="B6" s="328" t="inlineStr">
@@ -13291,22 +13271,6 @@
         <f>_xlfn.XLOOKUP('Consolidado- Comber'!$A$1&amp;"|"&amp;11,ListBox!$H:$H,ListBox!$A:$A,0,0)</f>
         <v>46311</v>
       </c>
-      <c r="P6" s="332">
-        <f>_xlfn.XLOOKUP('Consolidado- Comber'!$A$1&amp;"|"&amp;12,ListBox!$H:$H,ListBox!$A:$A,0,0)</f>
-        <v>46314</v>
-      </c>
-      <c r="Q6" s="332">
-        <f>_xlfn.XLOOKUP('Consolidado- Comber'!$A$1&amp;"|"&amp;13,ListBox!$H:$H,ListBox!$A:$A,0,0)</f>
-        <v>46315</v>
-      </c>
-      <c r="R6" s="332">
-        <f>_xlfn.XLOOKUP('Consolidado- Comber'!$A$1&amp;"|"&amp;14,ListBox!$H:$H,ListBox!$A:$A,0,0)</f>
-        <v>46316</v>
-      </c>
-      <c r="S6" s="332">
-        <f>_xlfn.XLOOKUP('Consolidado- Comber'!$A$1&amp;"|"&amp;15,ListBox!$H:$H,ListBox!$A:$A,0,0)</f>
-        <v>46317</v>
-      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="B7" s="330" t="inlineStr">
@@ -13362,22 +13326,6 @@
       <c r="O7" s="333" t="str">
         <f>LOWER(TEXT(O6,"ddd"))</f>
         <v>sex</v>
-      </c>
-      <c r="P7" s="333" t="str">
-        <f>LOWER(TEXT(P6,"ddd"))</f>
-        <v>seg</v>
-      </c>
-      <c r="Q7" s="333" t="str">
-        <f>LOWER(TEXT(Q6,"ddd"))</f>
-        <v>ter</v>
-      </c>
-      <c r="R7" s="333" t="str">
-        <f>LOWER(TEXT(R6,"ddd"))</f>
-        <v>qua</v>
-      </c>
-      <c r="S7" s="333" t="str">
-        <f>LOWER(TEXT(S6,"ddd"))</f>
-        <v>qui</v>
       </c>
     </row>
     <row r="8" ht="6" customHeight="1"/>
@@ -13404,10 +13352,6 @@
       <c r="M9" s="336"/>
       <c r="N9" s="336"/>
       <c r="O9" s="336"/>
-      <c r="P9" s="336"/>
-      <c r="Q9" s="336"/>
-      <c r="R9" s="336"/>
-      <c r="S9" s="336"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="337" t="inlineStr">
@@ -13436,10 +13380,6 @@
       <c r="M10" s="340"/>
       <c r="N10" s="340"/>
       <c r="O10" s="340"/>
-      <c r="P10" s="340"/>
-      <c r="Q10" s="340"/>
-      <c r="R10" s="340"/>
-      <c r="S10" s="340"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="337" t="inlineStr">
@@ -13468,10 +13408,6 @@
       <c r="M11" s="340"/>
       <c r="N11" s="340"/>
       <c r="O11" s="340"/>
-      <c r="P11" s="340"/>
-      <c r="Q11" s="340"/>
-      <c r="R11" s="340"/>
-      <c r="S11" s="340"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="B12" s="337" t="inlineStr">
@@ -13500,10 +13436,6 @@
       <c r="M12" s="340"/>
       <c r="N12" s="340"/>
       <c r="O12" s="340"/>
-      <c r="P12" s="340"/>
-      <c r="Q12" s="340"/>
-      <c r="R12" s="340"/>
-      <c r="S12" s="340"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="337" t="inlineStr">
@@ -13532,10 +13464,6 @@
       <c r="M13" s="340"/>
       <c r="N13" s="340"/>
       <c r="O13" s="340"/>
-      <c r="P13" s="340"/>
-      <c r="Q13" s="340"/>
-      <c r="R13" s="340"/>
-      <c r="S13" s="340"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="B14" s="341" t="inlineStr">
@@ -13560,10 +13488,6 @@
       <c r="M14" s="343"/>
       <c r="N14" s="343"/>
       <c r="O14" s="343"/>
-      <c r="P14" s="343"/>
-      <c r="Q14" s="343"/>
-      <c r="R14" s="343"/>
-      <c r="S14" s="343"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="337" t="inlineStr">
@@ -13592,10 +13516,6 @@
       <c r="M15" s="340"/>
       <c r="N15" s="340"/>
       <c r="O15" s="340"/>
-      <c r="P15" s="340"/>
-      <c r="Q15" s="340"/>
-      <c r="R15" s="340"/>
-      <c r="S15" s="340"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="B16" s="337" t="inlineStr">
@@ -13624,10 +13544,6 @@
       <c r="M16" s="340"/>
       <c r="N16" s="340"/>
       <c r="O16" s="340"/>
-      <c r="P16" s="340"/>
-      <c r="Q16" s="340"/>
-      <c r="R16" s="340"/>
-      <c r="S16" s="340"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="B17" s="345" t="inlineStr">
@@ -13652,10 +13568,6 @@
       <c r="M17" s="347"/>
       <c r="N17" s="347"/>
       <c r="O17" s="347"/>
-      <c r="P17" s="347"/>
-      <c r="Q17" s="347"/>
-      <c r="R17" s="347"/>
-      <c r="S17" s="347"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="B18" s="337" t="inlineStr">
@@ -13684,10 +13596,6 @@
       <c r="M18" s="340"/>
       <c r="N18" s="340"/>
       <c r="O18" s="340"/>
-      <c r="P18" s="340"/>
-      <c r="Q18" s="340"/>
-      <c r="R18" s="340"/>
-      <c r="S18" s="340"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="B19" s="337" t="inlineStr">
@@ -13716,10 +13624,6 @@
       <c r="M19" s="340"/>
       <c r="N19" s="340"/>
       <c r="O19" s="340"/>
-      <c r="P19" s="340"/>
-      <c r="Q19" s="340"/>
-      <c r="R19" s="340"/>
-      <c r="S19" s="340"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="B20" s="337" t="inlineStr">
@@ -13748,10 +13652,6 @@
       <c r="M20" s="340"/>
       <c r="N20" s="340"/>
       <c r="O20" s="340"/>
-      <c r="P20" s="340"/>
-      <c r="Q20" s="340"/>
-      <c r="R20" s="340"/>
-      <c r="S20" s="340"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="B21" s="337" t="inlineStr">
@@ -13780,10 +13680,6 @@
       <c r="M21" s="340"/>
       <c r="N21" s="340"/>
       <c r="O21" s="340"/>
-      <c r="P21" s="340"/>
-      <c r="Q21" s="340"/>
-      <c r="R21" s="340"/>
-      <c r="S21" s="340"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="B22" s="349" t="inlineStr">
@@ -13804,10 +13700,6 @@
       <c r="M22" s="351"/>
       <c r="N22" s="351"/>
       <c r="O22" s="351"/>
-      <c r="P22" s="351"/>
-      <c r="Q22" s="351"/>
-      <c r="R22" s="351"/>
-      <c r="S22" s="351"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="337" t="inlineStr">
@@ -13836,10 +13728,6 @@
       <c r="M23" s="340"/>
       <c r="N23" s="340"/>
       <c r="O23" s="340"/>
-      <c r="P23" s="340"/>
-      <c r="Q23" s="340"/>
-      <c r="R23" s="340"/>
-      <c r="S23" s="340"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="B24" s="353" t="inlineStr">
@@ -13864,10 +13752,6 @@
       <c r="M24" s="355"/>
       <c r="N24" s="355"/>
       <c r="O24" s="355"/>
-      <c r="P24" s="355"/>
-      <c r="Q24" s="355"/>
-      <c r="R24" s="355"/>
-      <c r="S24" s="355"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="337" t="inlineStr">
@@ -13900,15 +13784,11 @@
       <c r="M25" s="340"/>
       <c r="N25" s="340"/>
       <c r="O25" s="340"/>
-      <c r="P25" s="340"/>
-      <c r="Q25" s="340"/>
-      <c r="R25" s="340"/>
-      <c r="S25" s="340"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="B26" s="337" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apuração de PIS/COFINS</t>
+          <t xml:space="preserve">Apuração de PIS/COFINS (após o balancete)</t>
         </is>
       </c>
       <c r="C26" s="338" t="inlineStr">
@@ -13936,20 +13816,16 @@
           <t xml:space="preserve">···</t>
         </is>
       </c>
-      <c r="P26" s="360"/>
-      <c r="Q26" s="360"/>
-      <c r="R26" s="360"/>
-      <c r="S26" s="360"/>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="B27" s="361" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 · Contabilidade</t>
+          <t xml:space="preserve">6 · Contabilidade e balancete fechado</t>
         </is>
       </c>
       <c r="C27" s="362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Começa com as apurações; libera o PIS/COFINS ao ser entregue</t>
+          <t xml:space="preserve">Começa com as apurações; o balancete fechado (10º d.u.) libera o PIS/COFINS</t>
         </is>
       </c>
       <c r="D27" s="363"/>
@@ -13964,15 +13840,11 @@
       <c r="M27" s="363"/>
       <c r="N27" s="363"/>
       <c r="O27" s="363"/>
-      <c r="P27" s="363"/>
-      <c r="Q27" s="363"/>
-      <c r="R27" s="363"/>
-      <c r="S27" s="363"/>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="B28" s="337" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contabilidade</t>
+          <t xml:space="preserve">Contabilidade → balancete fechado</t>
         </is>
       </c>
       <c r="C28" s="338" t="inlineStr">
@@ -14000,67 +13872,38 @@
         </is>
       </c>
       <c r="O28" s="340"/>
-      <c r="P28" s="340"/>
-      <c r="Q28" s="340"/>
-      <c r="R28" s="340"/>
-      <c r="S28" s="340"/>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="337" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Balancete fechado</t>
-        </is>
-      </c>
-      <c r="C29" s="338" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Joyce · Equipe Contábil</t>
-        </is>
-      </c>
-      <c r="D29" s="340"/>
-      <c r="E29" s="340"/>
-      <c r="F29" s="340"/>
-      <c r="G29" s="340"/>
-      <c r="H29" s="340"/>
-      <c r="I29" s="340"/>
-      <c r="J29" s="340"/>
-      <c r="K29" s="340"/>
-      <c r="L29" s="340"/>
-      <c r="M29" s="340"/>
-      <c r="N29" s="340"/>
-      <c r="O29" s="340"/>
-      <c r="P29" s="340"/>
-      <c r="Q29" s="340"/>
-      <c r="R29" s="340"/>
-      <c r="S29" s="366" t="inlineStr">
-        <is>
-          <t xml:space="preserve">◆</t>
-        </is>
-      </c>
-    </row>
-    <row r="30"/>
-    <row r="31" ht="20" customHeight="1">
-      <c r="B31" s="367" t="inlineStr">
+    </row>
+    <row r="29"/>
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="367" t="inlineStr">
         <is>
           <t xml:space="preserve">LEGENDA</t>
         </is>
       </c>
-      <c r="C31" s="368" t="inlineStr">
+      <c r="C30" s="368" t="inlineStr">
         <is>
           <t xml:space="preserve">◆  entrega / prazo final (até 18:00)     ■  período de execução     ···  depende de etapa anterior (sem prazo fixo)</t>
         </is>
       </c>
     </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="B31" s="369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ordem do fluxo: áreas operacionais (último dia) → trava e validação fiscal (1º d.u.) → apurações, contabilidade e financeiro (2º d.u.) → folha (4º d.u.) → impostos (7º d.u.) → contabilidade / balancete fechado (10º d.u.) → PIS/COFINS.</t>
+        </is>
+      </c>
+    </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="369" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ordem do fluxo: áreas operacionais (último dia) → trava e validação fiscal (1º d.u.) → apurações, contabilidade e financeiro (2º d.u.) → folha (4º d.u.) → impostos (7º d.u.) → contabilidade (10º d.u.) → PIS/COFINS → balancete fechado (15º d.u.).</t>
+          <t xml:space="preserve">Impostos: entrega 5 dias úteis após o início das apurações (2º d.u. + 5 = 7º d.u.). PIS/COFINS só é apurado depois da contabilidade finalizada.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="369" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impostos: entrega 5 dias úteis após o início das apurações (2º d.u. + 5 = 7º d.u.). PIS/COFINS só é apurado depois da contabilidade finalizada.</t>
+          <t xml:space="preserve">Em paralelo de 02/10 a 15/10: apurações fiscais, contabilidade, financeiro/patrimônio (02/10) e folha (06/10). A contabilidade recebe a folha e os impostos.</t>
         </is>
       </c>
     </row>
@@ -14072,19 +13915,20 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="B2:S2"/>
-    <mergeCell ref="B3:S3"/>
-    <mergeCell ref="C9:S9"/>
-    <mergeCell ref="C14:S14"/>
-    <mergeCell ref="C17:S17"/>
-    <mergeCell ref="C22:S22"/>
-    <mergeCell ref="C24:S24"/>
-    <mergeCell ref="C27:S27"/>
-    <mergeCell ref="C31:S31"/>
-    <mergeCell ref="B32:S32"/>
-    <mergeCell ref="B33:S33"/>
-    <mergeCell ref="B34:S34"/>
+  <mergeCells count="13">
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="B3:O3"/>
+    <mergeCell ref="C9:O9"/>
+    <mergeCell ref="C14:O14"/>
+    <mergeCell ref="C17:O17"/>
+    <mergeCell ref="C22:O22"/>
+    <mergeCell ref="C24:O24"/>
+    <mergeCell ref="C27:O27"/>
+    <mergeCell ref="C30:O30"/>
+    <mergeCell ref="B31:O31"/>
+    <mergeCell ref="B32:O32"/>
+    <mergeCell ref="B33:O33"/>
+    <mergeCell ref="B34:O34"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToHeight="0"/>

</xml_diff>

<commit_message>
Novo fluxo: correções no 1º-2º d.u., processos paralelos a partir do 3º d.u.
- Financeiro, apurações e contabilidade iniciam no 3º d.u.
- Impostos no 8º d.u. (5 d.u. após início das apurações)
- PIS/COFINS finalizado em 16/10 (11º d.u.)
- Contabilidade até 20/10 (13º d.u.) com balancete fechado
- Imagem e aba Fluxo no Tempo atualizadas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0125feEMvz8hWRDaMuVf6tsQ
</commit_message>
<xml_diff>
--- a/12. Ficha de Controle Grupo Comber - SETEMBRO 2026.xlsx
+++ b/12. Ficha de Controle Grupo Comber - SETEMBRO 2026.xlsx
@@ -881,7 +881,7 @@
     <numFmt numFmtId="165" formatCode="h:mm"/>
     <numFmt numFmtId="190" formatCode="dd/mmm"/>
   </numFmts>
-  <fonts count="116" x14ac:knownFonts="1">
+  <fonts count="115" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1483,6 +1483,13 @@
     </font>
     <font>
       <b/>
+      <sz val="8"/>
+      <color rgb="FF255E8E"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="10"/>
       <color rgb="FF2E75B6"/>
       <name val="Aptos"/>
@@ -1577,19 +1584,6 @@
     </font>
     <font>
       <b/>
-      <sz val="8"/>
-      <color rgb="FF2F7D6E"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF2F7D6E"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="10"/>
       <color rgb="FF548235"/>
       <name val="Aptos"/>
@@ -1649,7 +1643,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="46">
+  <fills count="45">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1862,6 +1856,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFC1D1DF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF2E75B6"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1892,18 +1892,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDFEBE9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF2F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFCFDCC6"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1921,7 +1909,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="126">
+  <borders count="125">
     <border>
       <left/>
       <right/>
@@ -3033,6 +3021,19 @@
       <diagonal/>
     </border>
     <border>
+      <left style="hair">
+        <color rgb="FFD6DEE8"/>
+      </left>
+      <right style="hair">
+        <color rgb="FFD6DEE8"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color rgb="FFD6DEE8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
@@ -3179,32 +3180,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="hair">
-        <color rgb="FFD6DEE8"/>
-      </left>
-      <right style="hair">
-        <color rgb="FFD6DEE8"/>
-      </right>
-      <top/>
-      <bottom style="hair">
-        <color rgb="FFD6DEE8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color rgb="FFD6DEE8"/>
-      </left>
-      <right style="hair">
-        <color rgb="FFD6DEE8"/>
-      </right>
-      <top/>
-      <bottom style="hair">
-        <color rgb="FFD6DEE8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -3276,7 +3251,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="370">
+  <cellXfs count="369">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4255,8 +4230,8 @@
     <xf numFmtId="0" fontId="90" fillId="35" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="91" fillId="0" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="91" fillId="36" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="92" fillId="0" borderId="105" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -4264,11 +4239,11 @@
     <xf numFmtId="0" fontId="93" fillId="0" borderId="106" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="94" fillId="36" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="95" fillId="37" borderId="108" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="95" fillId="0" borderId="108" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="96" fillId="0" borderId="109" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -4276,11 +4251,11 @@
     <xf numFmtId="0" fontId="97" fillId="0" borderId="110" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="98" fillId="37" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="98" fillId="0" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="99" fillId="38" borderId="112" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="99" fillId="0" borderId="112" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="100" fillId="0" borderId="113" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -4288,20 +4263,20 @@
     <xf numFmtId="0" fontId="101" fillId="0" borderId="114" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="102" fillId="38" borderId="115" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="102" fillId="0" borderId="115" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="103" fillId="39" borderId="116" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="103" fillId="39" borderId="116" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="104" fillId="40" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="104" fillId="40" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="105" fillId="41" borderId="118" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="106" fillId="42" borderId="119" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="106" fillId="0" borderId="119" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="107" fillId="0" borderId="120" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -4309,25 +4284,22 @@
     <xf numFmtId="0" fontId="108" fillId="0" borderId="121" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="109" fillId="0" borderId="122" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="109" fillId="42" borderId="122" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="43" borderId="123" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="110" fillId="43" borderId="123" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="111" fillId="44" borderId="124" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="111" fillId="44" borderId="124" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="112" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="112" fillId="45" borderId="125" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="113" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="114" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="115" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -13119,14 +13091,14 @@
     <tabColor rgb="FF2E75B6"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:O34"/>
+  <dimension ref="B2:Q34"/>
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="2.5" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="15" width="9.5" customWidth="1"/>
-    <col min="16" max="16" width="2.5" customWidth="1"/>
+    <col min="4" max="17" width="9" customWidth="1"/>
+    <col min="18" max="18" width="2.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -13215,6 +13187,16 @@
           <t xml:space="preserve">11º d.u.</t>
         </is>
       </c>
+      <c r="P5" s="325" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12º d.u.</t>
+        </is>
+      </c>
+      <c r="Q5" s="325" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13º d.u.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="B6" s="328" t="inlineStr">
@@ -13271,6 +13253,14 @@
         <f>_xlfn.XLOOKUP('Consolidado- Comber'!$A$1&amp;"|"&amp;11,ListBox!$H:$H,ListBox!$A:$A,0,0)</f>
         <v>46311</v>
       </c>
+      <c r="P6" s="332">
+        <f>_xlfn.XLOOKUP('Consolidado- Comber'!$A$1&amp;"|"&amp;12,ListBox!$H:$H,ListBox!$A:$A,0,0)</f>
+        <v>46314</v>
+      </c>
+      <c r="Q6" s="332">
+        <f>_xlfn.XLOOKUP('Consolidado- Comber'!$A$1&amp;"|"&amp;13,ListBox!$H:$H,ListBox!$A:$A,0,0)</f>
+        <v>46315</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="B7" s="330" t="inlineStr">
@@ -13326,6 +13316,14 @@
       <c r="O7" s="333" t="str">
         <f>LOWER(TEXT(O6,"ddd"))</f>
         <v>sex</v>
+      </c>
+      <c r="P7" s="333" t="str">
+        <f>LOWER(TEXT(P6,"ddd"))</f>
+        <v>seg</v>
+      </c>
+      <c r="Q7" s="333" t="str">
+        <f>LOWER(TEXT(Q6,"ddd"))</f>
+        <v>ter</v>
       </c>
     </row>
     <row r="8" ht="6" customHeight="1"/>
@@ -13352,6 +13350,8 @@
       <c r="M9" s="336"/>
       <c r="N9" s="336"/>
       <c r="O9" s="336"/>
+      <c r="P9" s="336"/>
+      <c r="Q9" s="336"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="337" t="inlineStr">
@@ -13380,6 +13380,8 @@
       <c r="M10" s="340"/>
       <c r="N10" s="340"/>
       <c r="O10" s="340"/>
+      <c r="P10" s="340"/>
+      <c r="Q10" s="340"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="337" t="inlineStr">
@@ -13408,6 +13410,8 @@
       <c r="M11" s="340"/>
       <c r="N11" s="340"/>
       <c r="O11" s="340"/>
+      <c r="P11" s="340"/>
+      <c r="Q11" s="340"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="B12" s="337" t="inlineStr">
@@ -13436,6 +13440,8 @@
       <c r="M12" s="340"/>
       <c r="N12" s="340"/>
       <c r="O12" s="340"/>
+      <c r="P12" s="340"/>
+      <c r="Q12" s="340"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="337" t="inlineStr">
@@ -13464,16 +13470,18 @@
       <c r="M13" s="340"/>
       <c r="N13" s="340"/>
       <c r="O13" s="340"/>
+      <c r="P13" s="340"/>
+      <c r="Q13" s="340"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="B14" s="341" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 · Trava e validação fiscal</t>
+          <t xml:space="preserve">2 · Trava, validação fiscal e correções</t>
         </is>
       </c>
       <c r="C14" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sistema travado; o fiscal valida e as áreas corrigem no mesmo dia</t>
+          <t xml:space="preserve">Sistema travado no 1º d.u.; o time Comber corrige do 1º ao 2º d.u.</t>
         </is>
       </c>
       <c r="D14" s="343"/>
@@ -13488,6 +13496,8 @@
       <c r="M14" s="343"/>
       <c r="N14" s="343"/>
       <c r="O14" s="343"/>
+      <c r="P14" s="343"/>
+      <c r="Q14" s="343"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="337" t="inlineStr">
@@ -13516,11 +13526,13 @@
       <c r="M15" s="340"/>
       <c r="N15" s="340"/>
       <c r="O15" s="340"/>
+      <c r="P15" s="340"/>
+      <c r="Q15" s="340"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="B16" s="337" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dia das correções</t>
+          <t xml:space="preserve">Correções (time Comber)</t>
         </is>
       </c>
       <c r="C16" s="338" t="inlineStr">
@@ -13529,12 +13541,16 @@
         </is>
       </c>
       <c r="D16" s="340"/>
-      <c r="E16" s="344" t="inlineStr">
+      <c r="E16" s="345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">início</t>
+        </is>
+      </c>
+      <c r="F16" s="344" t="inlineStr">
         <is>
           <t xml:space="preserve">◆</t>
         </is>
       </c>
-      <c r="F16" s="340"/>
       <c r="G16" s="340"/>
       <c r="H16" s="340"/>
       <c r="I16" s="340"/>
@@ -13544,30 +13560,34 @@
       <c r="M16" s="340"/>
       <c r="N16" s="340"/>
       <c r="O16" s="340"/>
+      <c r="P16" s="340"/>
+      <c r="Q16" s="340"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="345" t="inlineStr">
+      <c r="B17" s="346" t="inlineStr">
         <is>
           <t xml:space="preserve">3 · Financeiro e patrimônio</t>
         </is>
       </c>
-      <c r="C17" s="346" t="inlineStr">
+      <c r="C17" s="347" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entregas no dia em que começam apurações e contabilidade</t>
+          <t xml:space="preserve">Entregas no dia em que começam apurações e contabilidade (3º d.u.)</t>
         </is>
       </c>
-      <c r="D17" s="347"/>
-      <c r="E17" s="347"/>
-      <c r="F17" s="347"/>
-      <c r="G17" s="347"/>
-      <c r="H17" s="347"/>
-      <c r="I17" s="347"/>
-      <c r="J17" s="347"/>
-      <c r="K17" s="347"/>
-      <c r="L17" s="347"/>
-      <c r="M17" s="347"/>
-      <c r="N17" s="347"/>
-      <c r="O17" s="347"/>
+      <c r="D17" s="348"/>
+      <c r="E17" s="348"/>
+      <c r="F17" s="348"/>
+      <c r="G17" s="348"/>
+      <c r="H17" s="348"/>
+      <c r="I17" s="348"/>
+      <c r="J17" s="348"/>
+      <c r="K17" s="348"/>
+      <c r="L17" s="348"/>
+      <c r="M17" s="348"/>
+      <c r="N17" s="348"/>
+      <c r="O17" s="348"/>
+      <c r="P17" s="348"/>
+      <c r="Q17" s="348"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="B18" s="337" t="inlineStr">
@@ -13582,12 +13602,12 @@
       </c>
       <c r="D18" s="340"/>
       <c r="E18" s="340"/>
-      <c r="F18" s="348" t="inlineStr">
+      <c r="F18" s="340"/>
+      <c r="G18" s="349" t="inlineStr">
         <is>
           <t xml:space="preserve">◆</t>
         </is>
       </c>
-      <c r="G18" s="340"/>
       <c r="H18" s="340"/>
       <c r="I18" s="340"/>
       <c r="J18" s="340"/>
@@ -13596,6 +13616,8 @@
       <c r="M18" s="340"/>
       <c r="N18" s="340"/>
       <c r="O18" s="340"/>
+      <c r="P18" s="340"/>
+      <c r="Q18" s="340"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="B19" s="337" t="inlineStr">
@@ -13610,12 +13632,12 @@
       </c>
       <c r="D19" s="340"/>
       <c r="E19" s="340"/>
-      <c r="F19" s="348" t="inlineStr">
+      <c r="F19" s="340"/>
+      <c r="G19" s="349" t="inlineStr">
         <is>
           <t xml:space="preserve">◆</t>
         </is>
       </c>
-      <c r="G19" s="340"/>
       <c r="H19" s="340"/>
       <c r="I19" s="340"/>
       <c r="J19" s="340"/>
@@ -13624,6 +13646,8 @@
       <c r="M19" s="340"/>
       <c r="N19" s="340"/>
       <c r="O19" s="340"/>
+      <c r="P19" s="340"/>
+      <c r="Q19" s="340"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="B20" s="337" t="inlineStr">
@@ -13638,12 +13662,12 @@
       </c>
       <c r="D20" s="340"/>
       <c r="E20" s="340"/>
-      <c r="F20" s="348" t="inlineStr">
+      <c r="F20" s="340"/>
+      <c r="G20" s="349" t="inlineStr">
         <is>
           <t xml:space="preserve">◆</t>
         </is>
       </c>
-      <c r="G20" s="340"/>
       <c r="H20" s="340"/>
       <c r="I20" s="340"/>
       <c r="J20" s="340"/>
@@ -13652,6 +13676,8 @@
       <c r="M20" s="340"/>
       <c r="N20" s="340"/>
       <c r="O20" s="340"/>
+      <c r="P20" s="340"/>
+      <c r="Q20" s="340"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="B21" s="337" t="inlineStr">
@@ -13666,12 +13692,12 @@
       </c>
       <c r="D21" s="340"/>
       <c r="E21" s="340"/>
-      <c r="F21" s="348" t="inlineStr">
+      <c r="F21" s="340"/>
+      <c r="G21" s="349" t="inlineStr">
         <is>
           <t xml:space="preserve">◆</t>
         </is>
       </c>
-      <c r="G21" s="340"/>
       <c r="H21" s="340"/>
       <c r="I21" s="340"/>
       <c r="J21" s="340"/>
@@ -13680,26 +13706,30 @@
       <c r="M21" s="340"/>
       <c r="N21" s="340"/>
       <c r="O21" s="340"/>
+      <c r="P21" s="340"/>
+      <c r="Q21" s="340"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="349" t="inlineStr">
+      <c r="B22" s="350" t="inlineStr">
         <is>
           <t xml:space="preserve">4 · Folha de pagamento</t>
         </is>
       </c>
-      <c r="C22" s="350"/>
-      <c r="D22" s="351"/>
-      <c r="E22" s="351"/>
-      <c r="F22" s="351"/>
-      <c r="G22" s="351"/>
-      <c r="H22" s="351"/>
-      <c r="I22" s="351"/>
-      <c r="J22" s="351"/>
-      <c r="K22" s="351"/>
-      <c r="L22" s="351"/>
-      <c r="M22" s="351"/>
-      <c r="N22" s="351"/>
-      <c r="O22" s="351"/>
+      <c r="C22" s="351"/>
+      <c r="D22" s="352"/>
+      <c r="E22" s="352"/>
+      <c r="F22" s="352"/>
+      <c r="G22" s="352"/>
+      <c r="H22" s="352"/>
+      <c r="I22" s="352"/>
+      <c r="J22" s="352"/>
+      <c r="K22" s="352"/>
+      <c r="L22" s="352"/>
+      <c r="M22" s="352"/>
+      <c r="N22" s="352"/>
+      <c r="O22" s="352"/>
+      <c r="P22" s="352"/>
+      <c r="Q22" s="352"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="337" t="inlineStr">
@@ -13716,7 +13746,7 @@
       <c r="E23" s="340"/>
       <c r="F23" s="340"/>
       <c r="G23" s="340"/>
-      <c r="H23" s="352" t="inlineStr">
+      <c r="H23" s="353" t="inlineStr">
         <is>
           <t xml:space="preserve">◆</t>
         </is>
@@ -13728,30 +13758,34 @@
       <c r="M23" s="340"/>
       <c r="N23" s="340"/>
       <c r="O23" s="340"/>
+      <c r="P23" s="340"/>
+      <c r="Q23" s="340"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="353" t="inlineStr">
+      <c r="B24" s="354" t="inlineStr">
         <is>
           <t xml:space="preserve">5 · Apurações fiscais</t>
         </is>
       </c>
-      <c r="C24" s="354" t="inlineStr">
+      <c r="C24" s="355" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entrega 5 dias úteis após o início das apurações</t>
+          <t xml:space="preserve">Impostos: entrega 5 dias úteis após o início das apurações</t>
         </is>
       </c>
-      <c r="D24" s="355"/>
-      <c r="E24" s="355"/>
-      <c r="F24" s="355"/>
-      <c r="G24" s="355"/>
-      <c r="H24" s="355"/>
-      <c r="I24" s="355"/>
-      <c r="J24" s="355"/>
-      <c r="K24" s="355"/>
-      <c r="L24" s="355"/>
-      <c r="M24" s="355"/>
-      <c r="N24" s="355"/>
-      <c r="O24" s="355"/>
+      <c r="D24" s="356"/>
+      <c r="E24" s="356"/>
+      <c r="F24" s="356"/>
+      <c r="G24" s="356"/>
+      <c r="H24" s="356"/>
+      <c r="I24" s="356"/>
+      <c r="J24" s="356"/>
+      <c r="K24" s="356"/>
+      <c r="L24" s="356"/>
+      <c r="M24" s="356"/>
+      <c r="N24" s="356"/>
+      <c r="O24" s="356"/>
+      <c r="P24" s="356"/>
+      <c r="Q24" s="356"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="337" t="inlineStr">
@@ -13766,29 +13800,31 @@
       </c>
       <c r="D25" s="340"/>
       <c r="E25" s="340"/>
-      <c r="F25" s="356" t="inlineStr">
+      <c r="F25" s="340"/>
+      <c r="G25" s="357" t="inlineStr">
         <is>
           <t xml:space="preserve">início</t>
         </is>
       </c>
-      <c r="G25" s="357"/>
-      <c r="H25" s="357"/>
-      <c r="I25" s="357"/>
-      <c r="J25" s="357"/>
-      <c r="K25" s="358" t="inlineStr">
+      <c r="H25" s="358"/>
+      <c r="I25" s="358"/>
+      <c r="J25" s="358"/>
+      <c r="K25" s="358"/>
+      <c r="L25" s="359" t="inlineStr">
         <is>
           <t xml:space="preserve">◆</t>
         </is>
       </c>
-      <c r="L25" s="340"/>
       <c r="M25" s="340"/>
       <c r="N25" s="340"/>
       <c r="O25" s="340"/>
+      <c r="P25" s="340"/>
+      <c r="Q25" s="340"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="B26" s="337" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apuração de PIS/COFINS (após o balancete)</t>
+          <t xml:space="preserve">PIS/COFINS finalizado</t>
         </is>
       </c>
       <c r="C26" s="338" t="inlineStr">
@@ -13806,40 +13842,40 @@
       <c r="K26" s="340"/>
       <c r="L26" s="340"/>
       <c r="M26" s="340"/>
-      <c r="N26" s="359" t="inlineStr">
+      <c r="N26" s="340"/>
+      <c r="O26" s="359" t="inlineStr">
         <is>
-          <t xml:space="preserve">após ▸</t>
+          <t xml:space="preserve">◆</t>
         </is>
       </c>
-      <c r="O26" s="360" t="inlineStr">
-        <is>
-          <t xml:space="preserve">···</t>
-        </is>
-      </c>
+      <c r="P26" s="340"/>
+      <c r="Q26" s="340"/>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="361" t="inlineStr">
+      <c r="B27" s="360" t="inlineStr">
         <is>
           <t xml:space="preserve">6 · Contabilidade e balancete fechado</t>
         </is>
       </c>
-      <c r="C27" s="362" t="inlineStr">
+      <c r="C27" s="361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Começa com as apurações; o balancete fechado (10º d.u.) libera o PIS/COFINS</t>
+          <t xml:space="preserve">Começa no 3º d.u. e termina com o balancete fechado</t>
         </is>
       </c>
-      <c r="D27" s="363"/>
-      <c r="E27" s="363"/>
-      <c r="F27" s="363"/>
-      <c r="G27" s="363"/>
-      <c r="H27" s="363"/>
-      <c r="I27" s="363"/>
-      <c r="J27" s="363"/>
-      <c r="K27" s="363"/>
-      <c r="L27" s="363"/>
-      <c r="M27" s="363"/>
-      <c r="N27" s="363"/>
-      <c r="O27" s="363"/>
+      <c r="D27" s="362"/>
+      <c r="E27" s="362"/>
+      <c r="F27" s="362"/>
+      <c r="G27" s="362"/>
+      <c r="H27" s="362"/>
+      <c r="I27" s="362"/>
+      <c r="J27" s="362"/>
+      <c r="K27" s="362"/>
+      <c r="L27" s="362"/>
+      <c r="M27" s="362"/>
+      <c r="N27" s="362"/>
+      <c r="O27" s="362"/>
+      <c r="P27" s="362"/>
+      <c r="Q27" s="362"/>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="B28" s="337" t="inlineStr">
@@ -13854,61 +13890,63 @@
       </c>
       <c r="D28" s="340"/>
       <c r="E28" s="340"/>
-      <c r="F28" s="364" t="inlineStr">
+      <c r="F28" s="340"/>
+      <c r="G28" s="363" t="inlineStr">
         <is>
           <t xml:space="preserve">início</t>
         </is>
       </c>
-      <c r="G28" s="365"/>
-      <c r="H28" s="365"/>
-      <c r="I28" s="365"/>
-      <c r="J28" s="365"/>
-      <c r="K28" s="365"/>
-      <c r="L28" s="365"/>
-      <c r="M28" s="365"/>
-      <c r="N28" s="366" t="inlineStr">
+      <c r="H28" s="364"/>
+      <c r="I28" s="364"/>
+      <c r="J28" s="364"/>
+      <c r="K28" s="364"/>
+      <c r="L28" s="364"/>
+      <c r="M28" s="364"/>
+      <c r="N28" s="364"/>
+      <c r="O28" s="364"/>
+      <c r="P28" s="364"/>
+      <c r="Q28" s="365" t="inlineStr">
         <is>
           <t xml:space="preserve">◆</t>
         </is>
       </c>
-      <c r="O28" s="340"/>
     </row>
     <row r="29"/>
     <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="367" t="inlineStr">
+      <c r="B30" s="366" t="inlineStr">
         <is>
           <t xml:space="preserve">LEGENDA</t>
         </is>
       </c>
-      <c r="C30" s="368" t="inlineStr">
+      <c r="C30" s="367" t="inlineStr">
         <is>
           <t xml:space="preserve">◆  entrega / prazo final (até 18:00)     ■  período de execução     ···  depende de etapa anterior (sem prazo fixo)</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="B31" s="369" t="inlineStr">
+      <c r="B31" s="368" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ordem do fluxo: áreas operacionais (último dia) → trava e validação fiscal (1º d.u.) → apurações, contabilidade e financeiro (2º d.u.) → folha (4º d.u.) → impostos (7º d.u.) → contabilidade / balancete fechado (10º d.u.) → PIS/COFINS.</t>
+          <t xml:space="preserve">Ordem do fluxo: áreas operacionais (último dia) → trava e validação fiscal (1º d.u.) → correções do time Comber (1º ao 2º d.u.) → apurações, contabilidade e financeiro (3º d.u.) → folha (4º d.u.) → impostos (8º d.u.) → PIS/COFINS (11º d.u.) → balancete fechado (13º d.u.).</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="B32" s="369" t="inlineStr">
+      <c r="B32" s="368" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impostos: entrega 5 dias úteis após o início das apurações (2º d.u. + 5 = 7º d.u.). PIS/COFINS só é apurado depois da contabilidade finalizada.</t>
+          <t xml:space="preserve">Impostos: entrega 5 dias úteis após o início das apurações (3º d.u. + 5 = 8º d.u.). PIS/COFINS finalizado no 11º d.u.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="B33" s="369" t="inlineStr">
+      <c r="B33" s="368" t="inlineStr">
         <is>
-          <t xml:space="preserve">Em paralelo de 02/10 a 15/10: apurações fiscais, contabilidade, financeiro/patrimônio (02/10) e folha (06/10). A contabilidade recebe a folha e os impostos.</t>
+          <t xml:space="preserve">Em paralelo do 3º ao 13º d.u.: apurações fiscais, contabilidade, financeiro/patrimônio (3º d.u.), folha (4º d.u.) e PIS/COFINS (11º d.u.). A contabilidade recebe a folha e os impostos.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="B34" s="369" t="inlineStr">
+      <c r="B34" s="368" t="inlineStr">
         <is>
           <t xml:space="preserve">Feriados e fins de semana não entram na contagem: as colunas mostram apenas dias úteis.</t>
         </is>
@@ -13916,19 +13954,19 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="B3:O3"/>
-    <mergeCell ref="C9:O9"/>
-    <mergeCell ref="C14:O14"/>
-    <mergeCell ref="C17:O17"/>
-    <mergeCell ref="C22:O22"/>
-    <mergeCell ref="C24:O24"/>
-    <mergeCell ref="C27:O27"/>
-    <mergeCell ref="C30:O30"/>
-    <mergeCell ref="B31:O31"/>
-    <mergeCell ref="B32:O32"/>
-    <mergeCell ref="B33:O33"/>
-    <mergeCell ref="B34:O34"/>
+    <mergeCell ref="B2:Q2"/>
+    <mergeCell ref="B3:Q3"/>
+    <mergeCell ref="C9:Q9"/>
+    <mergeCell ref="C14:Q14"/>
+    <mergeCell ref="C17:Q17"/>
+    <mergeCell ref="C22:Q22"/>
+    <mergeCell ref="C24:Q24"/>
+    <mergeCell ref="C27:Q27"/>
+    <mergeCell ref="C30:Q30"/>
+    <mergeCell ref="B31:Q31"/>
+    <mergeCell ref="B32:Q32"/>
+    <mergeCell ref="B33:Q33"/>
+    <mergeCell ref="B34:Q34"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToHeight="0"/>

</xml_diff>

<commit_message>
Mantém entrega dos impostos em 09/10 (7º d.u.)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0125feEMvz8hWRDaMuVf6tsQ
</commit_message>
<xml_diff>
--- a/12. Ficha de Controle Grupo Comber - SETEMBRO 2026.xlsx
+++ b/12. Ficha de Controle Grupo Comber - SETEMBRO 2026.xlsx
@@ -13769,7 +13769,7 @@
       </c>
       <c r="C24" s="355" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impostos: entrega 5 dias úteis após o início das apurações</t>
+          <t xml:space="preserve">Impostos entregues no 7º d.u.; PIS/COFINS no 11º d.u.</t>
         </is>
       </c>
       <c r="D24" s="356"/>
@@ -13809,12 +13809,12 @@
       <c r="H25" s="358"/>
       <c r="I25" s="358"/>
       <c r="J25" s="358"/>
-      <c r="K25" s="358"/>
-      <c r="L25" s="359" t="inlineStr">
+      <c r="K25" s="359" t="inlineStr">
         <is>
           <t xml:space="preserve">◆</t>
         </is>
       </c>
+      <c r="L25" s="340"/>
       <c r="M25" s="340"/>
       <c r="N25" s="340"/>
       <c r="O25" s="340"/>
@@ -13927,14 +13927,14 @@
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="368" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ordem do fluxo: áreas operacionais (último dia) → trava e validação fiscal (1º d.u.) → correções do time Comber (1º ao 2º d.u.) → apurações, contabilidade e financeiro (3º d.u.) → folha (4º d.u.) → impostos (8º d.u.) → PIS/COFINS (11º d.u.) → balancete fechado (13º d.u.).</t>
+          <t xml:space="preserve">Ordem do fluxo: áreas operacionais (último dia) → trava e validação fiscal (1º d.u.) → correções do time Comber (1º ao 2º d.u.) → apurações, contabilidade e financeiro (3º d.u.) → folha (4º d.u.) → impostos (7º d.u.) → PIS/COFINS (11º d.u.) → balancete fechado (13º d.u.).</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="368" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impostos: entrega 5 dias úteis após o início das apurações (3º d.u. + 5 = 8º d.u.). PIS/COFINS finalizado no 11º d.u.</t>
+          <t xml:space="preserve">Impostos (exceto PIS/COFINS) entregues no 7º d.u.; PIS/COFINS finalizado no 11º d.u.</t>
         </is>
       </c>
     </row>

</xml_diff>